<commit_message>
updated collaborations with cards css
</commit_message>
<xml_diff>
--- a/excels/collaboration_data.xlsx
+++ b/excels/collaboration_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\NITW-Transportation-Division-main\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC9779A2-E0BD-47FA-AEAA-35991C7AF33B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFA02BB1-AA83-4277-870D-8275D2235C18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Academic Collaboration" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="76">
   <si>
     <t>Project_Title</t>
   </si>
@@ -246,6 +246,9 @@
   </si>
   <si>
     <t>2022-08-15</t>
+  </si>
+  <si>
+    <t>Image</t>
   </si>
 </sst>
 </file>
@@ -585,13 +588,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -616,8 +625,11 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>8</v>
       </c>
@@ -640,7 +652,7 @@
         <v>1500000</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>14</v>
       </c>
@@ -666,7 +678,7 @@
         <v>2000000</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -689,7 +701,7 @@
         <v>1200000</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>26</v>
       </c>
@@ -715,7 +727,7 @@
         <v>1800000</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>32</v>
       </c>
@@ -738,7 +750,7 @@
         <v>1700000</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>36</v>
       </c>
@@ -761,6 +773,153 @@
         <v>20</v>
       </c>
       <c r="H7">
+        <v>1400000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
+        <v>13</v>
+      </c>
+      <c r="H8">
+        <v>1500000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" t="s">
+        <v>20</v>
+      </c>
+      <c r="H9">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
+        <v>25</v>
+      </c>
+      <c r="H10">
+        <v>1200000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B11" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11">
+        <v>1800000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12">
+        <v>1700000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" t="s">
+        <v>20</v>
+      </c>
+      <c r="H13">
         <v>1400000</v>
       </c>
     </row>
@@ -771,13 +930,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -802,8 +967,11 @@
       <c r="H1" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -826,7 +994,7 @@
         <v>2500000</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>50</v>
       </c>
@@ -852,7 +1020,7 @@
         <v>3000000</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>56</v>
       </c>
@@ -875,7 +1043,7 @@
         <v>2200000</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>60</v>
       </c>
@@ -901,7 +1069,7 @@
         <v>2700000</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>66</v>
       </c>
@@ -924,7 +1092,7 @@
         <v>2100000</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>70</v>
       </c>
@@ -947,6 +1115,153 @@
         <v>55</v>
       </c>
       <c r="H7">
+        <v>2600000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>45</v>
+      </c>
+      <c r="B8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D8" t="s">
+        <v>48</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" t="s">
+        <v>49</v>
+      </c>
+      <c r="H8">
+        <v>2500000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" t="s">
+        <v>53</v>
+      </c>
+      <c r="E9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F9" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" t="s">
+        <v>55</v>
+      </c>
+      <c r="H9">
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
+        <v>58</v>
+      </c>
+      <c r="D10" t="s">
+        <v>59</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
+        <v>49</v>
+      </c>
+      <c r="H10">
+        <v>2200000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D11" t="s">
+        <v>63</v>
+      </c>
+      <c r="E11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11">
+        <v>2700000</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>66</v>
+      </c>
+      <c r="B12" t="s">
+        <v>67</v>
+      </c>
+      <c r="C12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
+        <v>49</v>
+      </c>
+      <c r="H12">
+        <v>2100000</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C13" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" t="s">
+        <v>74</v>
+      </c>
+      <c r="F13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" t="s">
+        <v>55</v>
+      </c>
+      <c r="H13">
         <v>2600000</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated collaborations image data
</commit_message>
<xml_diff>
--- a/excels/collaboration_data.xlsx
+++ b/excels/collaboration_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEF4B8D8-1DF1-449B-AA0D-0C1F74DE1B41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E97078-6584-4348-A9D1-96E02C38115A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4005" yWindow="3825" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Academic Collaboration" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="33">
   <si>
     <t>Status</t>
   </si>
@@ -267,6 +267,12 @@
   </si>
   <si>
     <t>Organization_Name</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/PTV Vision, Germany.jpg</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/GeoVista, Hyderabad.jpg</t>
   </si>
 </sst>
 </file>
@@ -749,6 +755,9 @@
       <c r="B9" t="s">
         <v>2</v>
       </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
@@ -767,6 +776,9 @@
       </c>
       <c r="B11" t="s">
         <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -880,6 +892,9 @@
       <c r="B9" t="s">
         <v>2</v>
       </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
@@ -898,6 +913,9 @@
       </c>
       <c r="B11" t="s">
         <v>2</v>
+      </c>
+      <c r="C11" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
collaborations image error update
</commit_message>
<xml_diff>
--- a/excels/collaboration_data.xlsx
+++ b/excels/collaboration_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E97078-6584-4348-A9D1-96E02C38115A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B66134AD-A8FF-410E-8057-89CF413A272B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4005" yWindow="3825" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Academic Collaboration" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="31">
   <si>
     <t>Status</t>
   </si>
@@ -30,9 +30,6 @@
   </si>
   <si>
     <t>Completed</t>
-  </si>
-  <si>
-    <t>Image</t>
   </si>
   <si>
     <r>
@@ -85,7 +82,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">   </t>
+      <t xml:space="preserve">    </t>
     </r>
     <r>
       <rPr>
@@ -94,7 +91,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>Roads &amp; Buildings Dept., Govt. of AP</t>
+      <t>HUDA, Hyderabad</t>
     </r>
   </si>
   <si>
@@ -105,7 +102,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">  </t>
+      <t xml:space="preserve">    </t>
     </r>
     <r>
       <rPr>
@@ -114,7 +111,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>Panchayat Raj Engineering Dept., Govt. of AP</t>
+      <t>KUDA, Warangal</t>
     </r>
   </si>
   <si>
@@ -125,7 +122,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">    </t>
+      <t xml:space="preserve">     </t>
     </r>
     <r>
       <rPr>
@@ -134,7 +131,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>HUDA, Hyderabad</t>
+      <t>PTV Vision, Germany</t>
     </r>
   </si>
   <si>
@@ -145,7 +142,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">    </t>
+      <t xml:space="preserve">       </t>
     </r>
     <r>
       <rPr>
@@ -154,8 +151,53 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>KUDA, Warangal</t>
-    </r>
+      <t>C-DAC, Hyderabad</t>
+    </r>
+  </si>
+  <si>
+    <t>GeoVista, Hyderabad</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/Rites.jpg</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/Lea Associates.jpg</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/Singareni Colleries_Kothagudem.jpg</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/Roads &amp; Buildings Dept_Govt_of_AP.jpg</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/Panchayat Raj Engineering Dept_Govt_of_AP.jpg</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/HUDA.jpg</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/KUDA.jpg</t>
+  </si>
+  <si>
+    <t>Images/Collaborators/C-DAC_Hyderabad.jpg</t>
+  </si>
+  <si>
+    <t>C-DAC, Hyderabad</t>
+  </si>
+  <si>
+    <t>Singareni Colleries, Kothagudem</t>
+  </si>
+  <si>
+    <t>Roads &amp; Buildings Dept., Govt. of AP</t>
+  </si>
+  <si>
+    <t>Panchayat Raj Engineering Dept., Govt. of AP</t>
+  </si>
+  <si>
+    <t>HUDA, Hyderabad</t>
+  </si>
+  <si>
+    <t>KUDA, Warangal</t>
   </si>
   <si>
     <r>
@@ -165,7 +207,7 @@
         <rFont val="Times New Roman"/>
         <family val="1"/>
       </rPr>
-      <t xml:space="preserve">     </t>
+      <t xml:space="preserve"> </t>
     </r>
     <r>
       <rPr>
@@ -178,91 +220,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">       </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>C-DAC, Hyderabad</t>
-    </r>
-  </si>
-  <si>
-    <t>GeoVista, Hyderabad</t>
-  </si>
-  <si>
-    <t>Images/Collaborators/Rites.jpg</t>
-  </si>
-  <si>
-    <t>Images/Collaborators/Lea Associates.jpg</t>
-  </si>
-  <si>
-    <t>Images/Collaborators/Singareni Colleries_Kothagudem.jpg</t>
-  </si>
-  <si>
-    <t>Images/Collaborators/Roads &amp; Buildings Dept_Govt_of_AP.jpg</t>
-  </si>
-  <si>
-    <t>Images/Collaborators/Panchayat Raj Engineering Dept_Govt_of_AP.jpg</t>
-  </si>
-  <si>
-    <t>Images/Collaborators/HUDA.jpg</t>
-  </si>
-  <si>
-    <t>Images/Collaborators/KUDA.jpg</t>
-  </si>
-  <si>
-    <t>Images/Collaborators/C-DAC_Hyderabad.jpg</t>
-  </si>
-  <si>
-    <t>C-DAC, Hyderabad</t>
-  </si>
-  <si>
-    <t>Singareni Colleries, Kothagudem</t>
-  </si>
-  <si>
-    <t>Roads &amp; Buildings Dept., Govt. of AP</t>
-  </si>
-  <si>
-    <t>Panchayat Raj Engineering Dept., Govt. of AP</t>
-  </si>
-  <si>
-    <t>HUDA, Hyderabad</t>
-  </si>
-  <si>
-    <t>KUDA, Warangal</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>PTV Vision, Germany</t>
-    </r>
-  </si>
-  <si>
     <t>RITES, New Delhi</t>
   </si>
   <si>
@@ -273,6 +230,9 @@
   </si>
   <si>
     <t>Images/Collaborators/GeoVista, Hyderabad.jpg</t>
+  </si>
+  <si>
+    <t>Collab-Image</t>
   </si>
 </sst>
 </file>
@@ -326,7 +286,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -345,6 +305,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -662,123 +625,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
+      <c r="A5" s="7" t="s">
+        <v>21</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
+      <c r="A6" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
         <v>2</v>
       </c>
       <c r="C9" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -799,123 +762,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B4" t="s">
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B6" t="s">
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
         <v>28</v>
-      </c>
-      <c r="B9" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="B10" t="s">
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
         <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
collaborations data and css update
</commit_message>
<xml_diff>
--- a/excels/collaboration_data.xlsx
+++ b/excels/collaboration_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F068795-DE63-4BF6-8291-E5F45580E832}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4F10DE3-A459-45AA-8FA2-97E203113768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4005" yWindow="3825" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Academic Collaboration" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="25">
   <si>
     <t>Status</t>
   </si>
@@ -32,127 +32,7 @@
     <t>Completed</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>RITES, New Delhi</t>
-    </r>
-  </si>
-  <si>
     <t>Lea Associates, New Delhi</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Singareni Colleries, Kothagudem</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>HUDA, Hyderabad</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>KUDA, Warangal</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">     </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>PTV Vision, Germany</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="7"/>
-        <color theme="1"/>
-        <rFont val="Times New Roman"/>
-        <family val="1"/>
-      </rPr>
-      <t xml:space="preserve">       </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>C-DAC, Hyderabad</t>
-    </r>
   </si>
   <si>
     <t>GeoVista, Hyderabad</t>
@@ -286,12 +166,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -305,9 +182,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -614,7 +488,7 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="20.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="5" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -624,124 +498,124 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
-        <v>19</v>
+      <c r="A1" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>2</v>
-      </c>
-      <c r="C11" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -754,7 +628,7 @@
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.28515625" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="18.7109375" bestFit="1" customWidth="1"/>
@@ -762,123 +636,123 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
       </c>
       <c r="C1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C11" t="s">
         <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1</v>
-      </c>
-      <c r="C8" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" t="s">
-        <v>2</v>
-      </c>
-      <c r="C9" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C10" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>2</v>
-      </c>
-      <c r="C11" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>